<commit_message>
v21: expand authority evidence and harden release audit
</commit_message>
<xml_diff>
--- a/research/v21-seeded-documents/packs/antitrust/variant-01/documents/evidence-register.xlsx
+++ b/research/v21-seeded-documents/packs/antitrust/variant-01/documents/evidence-register.xlsx
@@ -16,8 +16,8 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Evidence Register'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Computation'!$A$1:$G$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'Computation'!$A$1:$G$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Instructions'!$A$1:$B$9</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Instructions'!$A$1:$B$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Instructions'!$A$1:$B$12</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Instructions'!$A$1:$B$12</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -807,7 +807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -901,29 +901,65 @@
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Forbidden phrase</t>
+          <t>Research authority</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>AUTO-CLOSE WITHOUT REVIEW</t>
+          <t>synthetic benchmark source; no external authority asserted</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Authority URL</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Research status</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Forbidden phrase</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>AUTO-CLOSE WITHOUT REVIEW</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Synthetic simulation only; attorney validation required before external use.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B9"/>
+  <autoFilter ref="A1:B12"/>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="1" fitToHeight="1" fitToWidth="1"/>

</xml_diff>